<commit_message>
Fix de plantilla de exportacion y el modulo de prefiniquitos
</commit_message>
<xml_diff>
--- a/backend/app/templates/excel/plantilla_de_sueldos_y_salarios.xlsx
+++ b/backend/app/templates/excel/plantilla_de_sueldos_y_salarios.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodnn\OneDrive\Desktop\Rodaltfl_dev_new\Proyects\plantillas_general\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rengifo\Desktop\Proyectos\sistema_de_boletas_de_pago-RengifoLtda\backend\app\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{495CC0BE-9BDE-4419-AE25-2D179E33C1CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284A849A-FDFD-4FD1-8E35-B13857E9491C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4AB49BEC-9586-4F07-8E7B-5982E757BCB2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4AB49BEC-9586-4F07-8E7B-5982E757BCB2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>N°</t>
   </si>
@@ -153,13 +153,22 @@
   </si>
   <si>
     <t>FIRMA</t>
+  </si>
+  <si>
+    <t>…............................................................................................................................................................</t>
+  </si>
+  <si>
+    <t>…..........................................................................................................</t>
+  </si>
+  <si>
+    <t>….................................................................................................</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,20 +177,50 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -198,7 +237,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -244,28 +283,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -298,84 +315,100 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -396,7 +429,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -712,310 +745,434 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92FEC31A-8724-4009-90BB-D87F2BDA40E5}">
-  <dimension ref="A2:X17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:X17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.109375" customWidth="1"/>
-    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" customWidth="1"/>
-    <col min="6" max="6" width="7.44140625" customWidth="1"/>
-    <col min="7" max="7" width="14.21875" customWidth="1"/>
-    <col min="8" max="8" width="13.88671875" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" customWidth="1"/>
-    <col min="12" max="12" width="11.5546875" customWidth="1"/>
-    <col min="13" max="13" width="11.77734375" customWidth="1"/>
-    <col min="14" max="14" width="11.109375" customWidth="1"/>
-    <col min="15" max="15" width="13.21875" customWidth="1"/>
-    <col min="16" max="16" width="12.44140625" customWidth="1"/>
-    <col min="18" max="18" width="10.6640625" customWidth="1"/>
-    <col min="19" max="19" width="12.77734375" customWidth="1"/>
-    <col min="20" max="20" width="8.21875" customWidth="1"/>
-    <col min="21" max="21" width="11.44140625" customWidth="1"/>
-    <col min="22" max="22" width="13.44140625" customWidth="1"/>
-    <col min="23" max="23" width="10.44140625" customWidth="1"/>
-    <col min="24" max="24" width="27.109375" customWidth="1"/>
+    <col min="10" max="10" width="9.5703125" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
+    <col min="14" max="14" width="11.140625" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" customWidth="1"/>
+    <col min="16" max="16" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" customWidth="1"/>
+    <col min="19" max="19" width="12.7109375" customWidth="1"/>
+    <col min="20" max="20" width="8.28515625" customWidth="1"/>
+    <col min="21" max="21" width="11.42578125" customWidth="1"/>
+    <col min="22" max="22" width="16.42578125" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" customWidth="1"/>
+    <col min="24" max="24" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:24" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+    </row>
+    <row r="2" spans="1:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15"/>
-      <c r="L2" s="26" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
       <c r="O2" s="9" t="s">
         <v>30</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="10"/>
-      <c r="R2" s="11"/>
-      <c r="U2" s="2" t="s">
+      <c r="R2" s="10"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="4"/>
-      <c r="W2" s="2" t="s">
+      <c r="V2" s="12"/>
+      <c r="W2" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="X2" s="4"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+      <c r="X2" s="12"/>
+    </row>
+    <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="17"/>
-      <c r="L3" s="26" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="8"/>
-    </row>
-    <row r="4" spans="1:24" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J5" s="25" t="s">
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+    </row>
+    <row r="4" spans="1:24" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+    </row>
+    <row r="5" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="J6" s="21" t="s">
+      <c r="K5" s="17"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="17"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="1"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="U6" s="21" t="s">
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="V6" s="1"/>
-      <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-    </row>
-    <row r="8" spans="1:24" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="27" t="s">
+      <c r="V6" s="15"/>
+      <c r="W6" s="15"/>
+      <c r="X6" s="15"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+    </row>
+    <row r="8" spans="1:24" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="28" t="s">
+      <c r="G8" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="28" t="s">
+      <c r="H8" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="28" t="s">
+      <c r="I8" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="28" t="s">
+      <c r="J8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="K8" s="28" t="s">
+      <c r="K8" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="28" t="s">
+      <c r="L8" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="28" t="s">
+      <c r="M8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N8" s="28" t="s">
+      <c r="N8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="O8" s="28" t="s">
+      <c r="O8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="P8" s="28" t="s">
+      <c r="P8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="28" t="s">
+      <c r="Q8" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="R8" s="28" t="s">
+      <c r="R8" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="S8" s="28" t="s">
+      <c r="S8" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="T8" s="28" t="s">
+      <c r="T8" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="U8" s="28" t="s">
+      <c r="U8" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="V8" s="28" t="s">
+      <c r="V8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="W8" s="28" t="s">
+      <c r="W8" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="X8" s="28" t="s">
+      <c r="X8" s="19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="28"/>
-      <c r="M9" s="28"/>
-      <c r="N9" s="28"/>
-      <c r="O9" s="28"/>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="28"/>
-      <c r="R9" s="28"/>
-      <c r="S9" s="28"/>
-      <c r="T9" s="28"/>
-      <c r="U9" s="28"/>
-      <c r="V9" s="28"/>
-      <c r="W9" s="28"/>
-      <c r="X9" s="28"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="28"/>
-      <c r="P10" s="28"/>
-      <c r="Q10" s="28"/>
-      <c r="R10" s="28"/>
-      <c r="S10" s="28"/>
-      <c r="T10" s="28"/>
-      <c r="U10" s="28"/>
-      <c r="V10" s="28"/>
-      <c r="W10" s="28"/>
-      <c r="X10" s="28"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A11" s="19">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
+      <c r="X10" s="19"/>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A11" s="20">
         <v>1</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="19"/>
-      <c r="O11" s="19"/>
-      <c r="P11" s="19"/>
-      <c r="Q11" s="19"/>
-      <c r="R11" s="19"/>
-      <c r="S11" s="19"/>
-      <c r="T11" s="19"/>
-      <c r="U11" s="19"/>
-      <c r="V11" s="19"/>
-      <c r="W11" s="19"/>
-      <c r="X11" s="19"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A12" s="19">
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
+      <c r="P11" s="20"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="20"/>
+      <c r="S11" s="20"/>
+      <c r="T11" s="20"/>
+      <c r="U11" s="20"/>
+      <c r="V11" s="20"/>
+      <c r="W11" s="20"/>
+      <c r="X11" s="20"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A12" s="20">
         <v>2</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
-      <c r="O12" s="19"/>
-      <c r="P12" s="19"/>
-      <c r="Q12" s="19"/>
-      <c r="R12" s="19"/>
-      <c r="S12" s="19"/>
-      <c r="T12" s="19"/>
-      <c r="U12" s="19"/>
-      <c r="V12" s="19"/>
-      <c r="W12" s="19"/>
-      <c r="X12" s="19"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A13" s="23" t="s">
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
+      <c r="M12" s="20"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="20"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="20"/>
+      <c r="S12" s="20"/>
+      <c r="T12" s="20"/>
+      <c r="U12" s="20"/>
+      <c r="V12" s="20"/>
+      <c r="W12" s="20"/>
+      <c r="X12" s="20"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A13" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="8"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="23"/>
       <c r="K13" s="24"/>
       <c r="L13" s="24"/>
       <c r="M13" s="24"/>
@@ -1031,69 +1188,137 @@
       <c r="W13" s="24"/>
       <c r="X13" s="24"/>
     </row>
-    <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
-    </row>
-    <row r="17" spans="4:21" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="21" t="s">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
+      <c r="V14" s="1"/>
+      <c r="W14" s="1"/>
+      <c r="X14" s="1"/>
+    </row>
+    <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="1"/>
+    </row>
+    <row r="16" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="S16" s="25"/>
+      <c r="T16" s="25"/>
+      <c r="U16" s="25"/>
+      <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
+      <c r="X16" s="1"/>
+    </row>
+    <row r="17" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="L17" s="21" t="s">
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="R17" s="22" t="s">
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="S17" s="18"/>
-      <c r="T17" s="18"/>
-      <c r="U17" s="18"/>
+      <c r="S17" s="27"/>
+      <c r="T17" s="27"/>
+      <c r="U17" s="27"/>
+      <c r="V17" s="1"/>
+      <c r="W17" s="1"/>
+      <c r="X17" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="D16:I16"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="R17:U17"/>
-    <mergeCell ref="O2:R2"/>
-    <mergeCell ref="O3:R3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="U6:X6"/>
-    <mergeCell ref="J5:O5"/>
-    <mergeCell ref="J6:O6"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:E3"/>
+  <mergeCells count="42">
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="D2:J2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
     <mergeCell ref="L2:N2"/>
-    <mergeCell ref="L3:N3"/>
     <mergeCell ref="S8:S10"/>
-    <mergeCell ref="T8:T10"/>
-    <mergeCell ref="U8:U10"/>
-    <mergeCell ref="V8:V10"/>
-    <mergeCell ref="W8:W10"/>
-    <mergeCell ref="X8:X10"/>
     <mergeCell ref="M8:M10"/>
     <mergeCell ref="N8:N10"/>
     <mergeCell ref="O8:O10"/>
@@ -1105,14 +1330,26 @@
     <mergeCell ref="I8:I10"/>
     <mergeCell ref="J8:J10"/>
     <mergeCell ref="K8:K10"/>
+    <mergeCell ref="R17:U17"/>
+    <mergeCell ref="U6:X6"/>
+    <mergeCell ref="J5:O5"/>
+    <mergeCell ref="J6:O6"/>
+    <mergeCell ref="T8:T10"/>
+    <mergeCell ref="U8:U10"/>
+    <mergeCell ref="V8:V10"/>
+    <mergeCell ref="W8:W10"/>
+    <mergeCell ref="X8:X10"/>
     <mergeCell ref="L8:L10"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
     <mergeCell ref="F8:F10"/>
+    <mergeCell ref="R16:U16"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="D16:I16"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="L16:O16"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.74803149606299213" bottom="0.19685039370078741" header="0.19685039370078741" footer="0.19685039370078741"/>
+  <pageSetup scale="44" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>